<commit_message>
Se añaden los cálculos de los costos de producción del proyecto
</commit_message>
<xml_diff>
--- a/CalculoTiempoCosto.xlsx
+++ b/CalculoTiempoCosto.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mario\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni\7mo semestre\Arquitectura e ingenieria de software\AEIDS_Practica1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A63F0AB3-8134-448D-AE4B-D7CB144F017C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80E5909E-A803-44FF-8D58-F3B891FEF1E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19320" yWindow="3015" windowWidth="19440" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Método de Estimación Puntos CU" sheetId="1" r:id="rId1"/>
@@ -2171,11 +2171,12 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
     <col min="3" max="3" width="13.5703125" style="74" customWidth="1"/>
     <col min="5" max="5" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
@@ -2240,6 +2241,7 @@
         <f t="shared" ref="I3:I10" si="2">+G3/H3</f>
         <v>18.242721874999997</v>
       </c>
+      <c r="K3" s="74"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="20" t="s">
@@ -2455,7 +2457,7 @@
       </c>
       <c r="B13" s="86">
         <f>+K37</f>
-        <v>510796.21249999991</v>
+        <v>1021592.4249999998</v>
       </c>
       <c r="E13" s="89" t="s">
         <v>67</v>
@@ -2473,7 +2475,7 @@
       </c>
       <c r="B14" s="80">
         <f>+K48</f>
-        <v>145941.77499999997</v>
+        <v>291883.54999999993</v>
       </c>
       <c r="E14" s="84" t="s">
         <v>75</v>
@@ -2503,7 +2505,7 @@
       </c>
       <c r="B15" s="80">
         <f>SUM(B11:B14)</f>
-        <v>955462.55820312467</v>
+        <v>1612200.5457031247</v>
       </c>
       <c r="E15" s="80">
         <f>+$C$3</f>
@@ -3024,11 +3026,11 @@
         <v>6.3849526562499985</v>
       </c>
       <c r="J37" s="80">
-        <v>40000</v>
+        <v>80000</v>
       </c>
       <c r="K37" s="80">
         <f>+J37*H37*I37</f>
-        <v>510796.21249999991</v>
+        <v>1021592.4249999998</v>
       </c>
     </row>
     <row r="38" spans="5:11" x14ac:dyDescent="0.2">
@@ -3051,11 +3053,11 @@
         <v>4.2566351041666657</v>
       </c>
       <c r="J38" s="80">
-        <v>40000</v>
+        <v>80000</v>
       </c>
       <c r="K38" s="80">
         <f t="shared" ref="K38:K44" si="14">+J38*H38*I38</f>
-        <v>510796.21249999991</v>
+        <v>1021592.4249999998</v>
       </c>
     </row>
     <row r="39" spans="5:11" x14ac:dyDescent="0.2">
@@ -3078,11 +3080,11 @@
         <v>3.1924763281249993</v>
       </c>
       <c r="J39" s="80">
-        <v>40000</v>
+        <v>80000</v>
       </c>
       <c r="K39" s="80">
         <f t="shared" si="14"/>
-        <v>510796.21249999991</v>
+        <v>1021592.4249999998</v>
       </c>
     </row>
     <row r="40" spans="5:11" x14ac:dyDescent="0.2">
@@ -3105,11 +3107,11 @@
         <v>2.5539810624999992</v>
       </c>
       <c r="J40" s="80">
-        <v>40000</v>
+        <v>80000</v>
       </c>
       <c r="K40" s="80">
         <f t="shared" si="14"/>
-        <v>510796.21249999985</v>
+        <v>1021592.4249999997</v>
       </c>
     </row>
     <row r="41" spans="5:11" x14ac:dyDescent="0.2">
@@ -3132,11 +3134,11 @@
         <v>2.1283175520833328</v>
       </c>
       <c r="J41" s="80">
-        <v>40000</v>
+        <v>80000</v>
       </c>
       <c r="K41" s="80">
         <f t="shared" si="14"/>
-        <v>510796.21249999991</v>
+        <v>1021592.4249999998</v>
       </c>
     </row>
     <row r="42" spans="5:11" x14ac:dyDescent="0.2">
@@ -3159,11 +3161,11 @@
         <v>1.8242721874999996</v>
       </c>
       <c r="J42" s="80">
-        <v>40000</v>
+        <v>80000</v>
       </c>
       <c r="K42" s="80">
         <f t="shared" si="14"/>
-        <v>510796.21249999991</v>
+        <v>1021592.4249999998</v>
       </c>
     </row>
     <row r="43" spans="5:11" x14ac:dyDescent="0.2">
@@ -3186,11 +3188,11 @@
         <v>1.5962381640624996</v>
       </c>
       <c r="J43" s="80">
-        <v>40000</v>
+        <v>80000</v>
       </c>
       <c r="K43" s="80">
         <f t="shared" si="14"/>
-        <v>510796.21249999991</v>
+        <v>1021592.4249999998</v>
       </c>
     </row>
     <row r="44" spans="5:11" x14ac:dyDescent="0.2">
@@ -3213,11 +3215,11 @@
         <v>1.4188783680555552</v>
       </c>
       <c r="J44" s="80">
-        <v>40000</v>
+        <v>80000</v>
       </c>
       <c r="K44" s="80">
         <f t="shared" si="14"/>
-        <v>510796.21249999991</v>
+        <v>1021592.4249999998</v>
       </c>
     </row>
     <row r="46" spans="5:11" x14ac:dyDescent="0.2">
@@ -3274,11 +3276,11 @@
         <v>3.6485443749999993</v>
       </c>
       <c r="J48" s="80">
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="K48" s="80">
         <f>+J48*H48*I48</f>
-        <v>145941.77499999997</v>
+        <v>291883.54999999993</v>
       </c>
     </row>
     <row r="49" spans="5:11" x14ac:dyDescent="0.2">
@@ -3301,11 +3303,11 @@
         <v>2.432362916666666</v>
       </c>
       <c r="J49" s="80">
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="K49" s="80">
         <f t="shared" ref="K49:K55" si="18">+J49*H49*I49</f>
-        <v>145941.77499999997</v>
+        <v>291883.54999999993</v>
       </c>
     </row>
     <row r="50" spans="5:11" x14ac:dyDescent="0.2">
@@ -3328,11 +3330,11 @@
         <v>1.8242721874999996</v>
       </c>
       <c r="J50" s="80">
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="K50" s="80">
         <f t="shared" si="18"/>
-        <v>145941.77499999997</v>
+        <v>291883.54999999993</v>
       </c>
     </row>
     <row r="51" spans="5:11" x14ac:dyDescent="0.2">
@@ -3355,11 +3357,11 @@
         <v>1.4594177499999996</v>
       </c>
       <c r="J51" s="80">
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="K51" s="80">
         <f t="shared" si="18"/>
-        <v>145941.77499999997</v>
+        <v>291883.54999999993</v>
       </c>
     </row>
     <row r="52" spans="5:11" x14ac:dyDescent="0.2">
@@ -3382,11 +3384,11 @@
         <v>1.216181458333333</v>
       </c>
       <c r="J52" s="80">
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="K52" s="80">
         <f t="shared" si="18"/>
-        <v>145941.77499999997</v>
+        <v>291883.54999999993</v>
       </c>
     </row>
     <row r="53" spans="5:11" x14ac:dyDescent="0.2">
@@ -3409,11 +3411,11 @@
         <v>1.0424412499999998</v>
       </c>
       <c r="J53" s="80">
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="K53" s="80">
         <f t="shared" si="18"/>
-        <v>145941.77499999997</v>
+        <v>291883.54999999993</v>
       </c>
     </row>
     <row r="54" spans="5:11" x14ac:dyDescent="0.2">
@@ -3436,11 +3438,11 @@
         <v>0.91213609374999982</v>
       </c>
       <c r="J54" s="80">
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="K54" s="80">
         <f t="shared" si="18"/>
-        <v>145941.77499999997</v>
+        <v>291883.54999999993</v>
       </c>
     </row>
     <row r="55" spans="5:11" x14ac:dyDescent="0.2">
@@ -3463,11 +3465,11 @@
         <v>0.81078763888888872</v>
       </c>
       <c r="J55" s="80">
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="K55" s="80">
         <f t="shared" si="18"/>
-        <v>145941.77499999997</v>
+        <v>291883.54999999993</v>
       </c>
     </row>
   </sheetData>

</xml_diff>